<commit_message>
Finished GV function scoring
</commit_message>
<xml_diff>
--- a/03_csf_scoring_workbook.xlsx
+++ b/03_csf_scoring_workbook.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="425">
   <si>
     <t>This document was exported from Numbers.  Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -479,12 +479,18 @@
     <t>The cybersecurity risk management strategy is reviewed and adjusted to ensure coverage of organizational requirements and risks</t>
   </si>
   <si>
+    <t>Strategic adjustments observable in response to changing requirements: FTC Safeguards Rule compliance project, SOC 2 Type II push driven by capital partner expectations, increased board attention following industry breaches. However, no documented strategy review process exists. Adjustments are reactive and project-based rather than emerging from a structured review of coverage gaps.</t>
+  </si>
+  <si>
     <t>GV.OV-03</t>
   </si>
   <si>
     <t>Organizational cybersecurity risk management performance is evaluated and reviewed for adjustments needed</t>
   </si>
   <si>
+    <t>Annual Board Audit Committee cybersecurity review provides limited program performance oversight. No documented metrics or formal performance evaluation framework mentioned in source documents — assumed absent given overall program maturity. Adjustments to program direction happen reactively to incidents or audit findings rather than from systematic performance data.</t>
+  </si>
+  <si>
     <t>Cybersecurity Supply Chain Risk Management</t>
   </si>
   <si>
@@ -497,58 +503,112 @@
     <t>A C-SCRM program, strategy, objectives, policies, and processes are established and agreed to by stakeholders</t>
   </si>
   <si>
+    <t>No formal C-SCRM program, strategy, or documented objectives exist. Legal performs ad hoc security diligence during contracting, but this is contract review activity rather than supply chain risk management. Vendor Management Policy drafted but not approved. No centralized vendor inventory, vendors fragmented across bill.com (finance), legal Google Sheet, and DocuSign CLM with no master view. No stakeholder-agreed C-SCRM framework exists.</t>
+  </si>
+  <si>
     <t>GV.SC-02</t>
   </si>
   <si>
     <t>Cybersecurity roles and responsibilities for suppliers, customers, and partners are established, communicated, and coordinated</t>
   </si>
   <si>
+    <t>No defined cybersecurity roles and responsibilities exist between MBC and its third parties. Legal performs ad hoc vendor diligence during contracting without consistent InfoSec involvement. Vendor Management Policy drafted but not approved. No security points of contact, incident notification protocols, or shared responsibility frameworks documented for critical integrations (Plaid, credit bureaus, CoreLogic, Black Knight, Salesforce). Customer-facing security responsibilities (borrower portal users) not communicated. Capital partner relationships involve partners imposing requirements on MBC (SOC 2 Type II requests) rather than coordinated cybersecurity role definition.</t>
+  </si>
+  <si>
     <t>GV.SC-03</t>
   </si>
   <si>
     <t>C-SCRM is integrated into cybersecurity and enterprise risk management, risk assessment, and improvement processes</t>
   </si>
   <si>
+    <t>No integration of C-SCRM into broader risk processes — primarily because C-SCRM doesn't exist as a formal program and ERM doesn't exist at MBC at all (per GV.RM-03). Vendor risk is not represented in the informal Notion security risk list. Vendor diligence sits in Legal during contracting, disconnected from any risk assessment process. No improvement cycle exists where vendor risks would surface and drive program adjustments.</t>
+  </si>
+  <si>
     <t>GV.SC-04</t>
   </si>
   <si>
     <t>Suppliers are known and prioritized by criticality</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <rFont val="Times Roman"/>
+      </rPr>
+      <t>No vendor inventory exists in any central system; vendors are tracked in finance (</t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="12"/>
+        <color indexed="11"/>
+        <rFont val="Times Roman"/>
+      </rPr>
+      <t>bill.com</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color indexed="8"/>
+        <rFont val="Times Roman"/>
+      </rPr>
+      <t>), legal (a Google Sheet), and procurement (DocuSign CLM) without a master view. No vendor tiering by criticality. Part of broader gap: no formal C-SCRM program.</t>
+    </r>
+  </si>
+  <si>
     <t>GV.SC-05</t>
   </si>
   <si>
     <t>Requirements to address cybersecurity risks in supply chains are established, prioritized, and integrated into contracts</t>
   </si>
   <si>
+    <t>No standard cybersecurity contractual requirements established for vendor agreements. Vendor Management Policy is drafted but not approved, so no required contract clauses are mandated. Legal performs ad hoc security questionnaires during contracting but completion is inconsistent and not tied to contractual security commitments. No prioritization framework exists to determine which vendors require what level of contractual security obligations. Part of broader gap: no formal C-SCRM program.</t>
+  </si>
+  <si>
     <t>GV.SC-06</t>
   </si>
   <si>
     <t>Planning and due diligence are performed to reduce risks before entering into supplier or other third-party relationships</t>
   </si>
   <si>
+    <t>No pre-engagement security due diligence framework exists. Security assessment happens during contracting (after vendor selection) rather than as part of pre-relationship evaluation. Security questionnaires requested for some vendors handling PII but completion is inconsistent and not gating to contract execution. No documented due diligence checklist, required artifacts, or risk acceptance authority defined before vendor relationships are entered. Part of broader gap: no formal C-SCRM program.</t>
+  </si>
+  <si>
     <t>GV.SC-07</t>
   </si>
   <si>
     <t>Risks posed by suppliers, their products/services, and third parties are recorded, prioritized, assessed, responded to, and monitored</t>
   </si>
   <si>
+    <t>No ongoing vendor risk management process exists. Vendor risks are not recorded in any central register; the informal Notion security risk list (~30 items) is not vendor-focused. No prioritization, periodic reassessment, or documented response process for vendor-related risks across the relationship lifecycle. Vendor security assessment happens only at contracting, then is not revisited. Part of broader gap: no formal C-SCRM program.</t>
+  </si>
+  <si>
     <t>GV.SC-08</t>
   </si>
   <si>
     <t>Relevant suppliers and third parties are included in incident planning, response, and recovery activities</t>
   </si>
   <si>
+    <t>No process to include third parties in incident planning, response, or recovery activities. IR plan references a Mandiant retainer for major incident support but the retainer is currently expired and unrenewed. No suppliers participate in tabletop exercises (none performed in 12+ months regardless). No contractual incident notification requirements for vendors documented. External notification process exists for regulators and capital partners but is one-way notification, not collaborative incident coordination.</t>
+  </si>
+  <si>
     <t>GV.SC-09</t>
   </si>
   <si>
     <t>Supply chain security practices are integrated into cybersecurity and ERM programs, with performance monitored across product/service lifecycles</t>
   </si>
   <si>
+    <t>No C-SCRM program exists and no ERM process exists at MBC, so integration of supply chain security into either cannot occur. Vendor security performance is not monitored across the technology lifecycle — no documented checks at vendor selection, deployment (the addendum notes three recent SaaS additions not yet in Okta), ongoing operation, or vendor offboarding. No metrics on supply chain security performance. Part of broader gap: no formal C-SCRM program.</t>
+  </si>
+  <si>
     <t>GV.SC-10</t>
   </si>
   <si>
     <t>C-SCRM plans include provisions for activities that occur after the conclusion of a partnership or service agreement</t>
+  </si>
+  <si>
+    <t>No vendor offboarding or relationship-conclusion provisions documented. Source documents are silent on data return/destruction requirements, access and credential revocation processes, or contract close-out procedures when vendor relationships end. Vendor Management Policy (drafted but unapproved) does not specify end-of-relationship security obligations. Given the absence of a formal C-SCRM program, offboarding provisions are assumed absent. Part of broader gap: no formal C-SCRM program.</t>
   </si>
   <si>
     <t>Identify</t>
@@ -1811,11 +1871,11 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="9" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="8" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3167,7 +3227,7 @@
     </row>
     <row r="15">
       <c r="B15" t="s" s="3">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -3178,12 +3238,12 @@
         <v>5</v>
       </c>
       <c r="D16" t="s" s="5">
-        <v>354</v>
+        <v>366</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="s" s="3">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -3194,7 +3254,7 @@
         <v>5</v>
       </c>
       <c r="D18" t="s" s="5">
-        <v>384</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -4414,12 +4474,19 @@
       <c r="F21" t="s" s="17">
         <v>137</v>
       </c>
-      <c r="G21" s="44"/>
-      <c r="H21" s="44"/>
-      <c r="I21" t="str" s="44" cm="1">
+      <c r="G21" s="41">
+        <v>2</v>
+      </c>
+      <c r="H21" s="41">
+        <v>3</v>
+      </c>
+      <c r="I21" s="42" cm="1">
         <f t="array" ref="I21">IF(AND(ISNUMBER(G21),ISNUMBER(H21)),H21-G21,"")</f>
-      </c>
-      <c r="J21" s="46"/>
+        <v>1</v>
+      </c>
+      <c r="J21" t="s" s="43">
+        <v>138</v>
+      </c>
       <c r="K21" s="42"/>
       <c r="L21" s="44"/>
     </row>
@@ -4437,17 +4504,24 @@
         <v>132</v>
       </c>
       <c r="E22" t="s" s="40">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F22" t="s" s="17">
-        <v>139</v>
-      </c>
-      <c r="G22" s="44"/>
-      <c r="H22" s="44"/>
-      <c r="I22" t="str" s="44" cm="1">
+        <v>140</v>
+      </c>
+      <c r="G22" s="41">
+        <v>2</v>
+      </c>
+      <c r="H22" s="41">
+        <v>3</v>
+      </c>
+      <c r="I22" s="42" cm="1">
         <f t="array" ref="I22">IF(AND(ISNUMBER(G22),ISNUMBER(H22)),H22-G22,"")</f>
-      </c>
-      <c r="J22" s="46"/>
+        <v>1</v>
+      </c>
+      <c r="J22" t="s" s="43">
+        <v>141</v>
+      </c>
       <c r="K22" s="42"/>
       <c r="L22" s="44"/>
     </row>
@@ -4459,23 +4533,30 @@
         <v>68</v>
       </c>
       <c r="C23" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D23" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E23" t="s" s="40">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F23" t="s" s="17">
-        <v>143</v>
-      </c>
-      <c r="G23" s="44"/>
-      <c r="H23" s="44"/>
-      <c r="I23" t="str" s="44" cm="1">
+        <v>145</v>
+      </c>
+      <c r="G23" s="41">
+        <v>1</v>
+      </c>
+      <c r="H23" s="41">
+        <v>3</v>
+      </c>
+      <c r="I23" s="42" cm="1">
         <f t="array" ref="I23">IF(AND(ISNUMBER(G23),ISNUMBER(H23)),H23-G23,"")</f>
-      </c>
-      <c r="J23" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J23" t="s" s="43">
+        <v>146</v>
+      </c>
       <c r="K23" s="42"/>
       <c r="L23" s="44"/>
     </row>
@@ -4487,23 +4568,30 @@
         <v>68</v>
       </c>
       <c r="C24" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D24" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E24" t="s" s="40">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F24" t="s" s="17">
-        <v>145</v>
-      </c>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44"/>
-      <c r="I24" t="str" s="44" cm="1">
+        <v>148</v>
+      </c>
+      <c r="G24" s="41">
+        <v>1</v>
+      </c>
+      <c r="H24" s="41">
+        <v>3</v>
+      </c>
+      <c r="I24" s="42" cm="1">
         <f t="array" ref="I24">IF(AND(ISNUMBER(G24),ISNUMBER(H24)),H24-G24,"")</f>
-      </c>
-      <c r="J24" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J24" t="s" s="43">
+        <v>149</v>
+      </c>
       <c r="K24" s="42"/>
       <c r="L24" s="44"/>
     </row>
@@ -4515,23 +4603,30 @@
         <v>68</v>
       </c>
       <c r="C25" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D25" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E25" t="s" s="40">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="F25" t="s" s="17">
-        <v>147</v>
-      </c>
-      <c r="G25" s="44"/>
-      <c r="H25" s="44"/>
-      <c r="I25" t="str" s="44" cm="1">
+        <v>151</v>
+      </c>
+      <c r="G25" s="41">
+        <v>1</v>
+      </c>
+      <c r="H25" s="41">
+        <v>3</v>
+      </c>
+      <c r="I25" s="42" cm="1">
         <f t="array" ref="I25">IF(AND(ISNUMBER(G25),ISNUMBER(H25)),H25-G25,"")</f>
-      </c>
-      <c r="J25" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J25" t="s" s="43">
+        <v>152</v>
+      </c>
       <c r="K25" s="42"/>
       <c r="L25" s="44"/>
     </row>
@@ -4543,23 +4638,30 @@
         <v>68</v>
       </c>
       <c r="C26" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D26" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E26" t="s" s="40">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F26" t="s" s="17">
-        <v>149</v>
-      </c>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" t="str" s="44" cm="1">
+        <v>154</v>
+      </c>
+      <c r="G26" s="41">
+        <v>1</v>
+      </c>
+      <c r="H26" s="41">
+        <v>3</v>
+      </c>
+      <c r="I26" s="42" cm="1">
         <f t="array" ref="I26">IF(AND(ISNUMBER(G26),ISNUMBER(H26)),H26-G26,"")</f>
-      </c>
-      <c r="J26" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J26" t="s" s="45">
+        <v>155</v>
+      </c>
       <c r="K26" s="42"/>
       <c r="L26" s="44"/>
     </row>
@@ -4571,23 +4673,30 @@
         <v>68</v>
       </c>
       <c r="C27" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D27" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E27" t="s" s="40">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F27" t="s" s="17">
-        <v>151</v>
-      </c>
-      <c r="G27" s="44"/>
-      <c r="H27" s="44"/>
-      <c r="I27" t="str" s="44" cm="1">
+        <v>157</v>
+      </c>
+      <c r="G27" s="41">
+        <v>1</v>
+      </c>
+      <c r="H27" s="41">
+        <v>3</v>
+      </c>
+      <c r="I27" s="42" cm="1">
         <f t="array" ref="I27">IF(AND(ISNUMBER(G27),ISNUMBER(H27)),H27-G27,"")</f>
-      </c>
-      <c r="J27" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J27" t="s" s="43">
+        <v>158</v>
+      </c>
       <c r="K27" s="42"/>
       <c r="L27" s="44"/>
     </row>
@@ -4599,23 +4708,30 @@
         <v>68</v>
       </c>
       <c r="C28" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D28" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E28" t="s" s="40">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="F28" t="s" s="17">
-        <v>153</v>
-      </c>
-      <c r="G28" s="44"/>
-      <c r="H28" s="44"/>
-      <c r="I28" t="str" s="44" cm="1">
+        <v>160</v>
+      </c>
+      <c r="G28" s="41">
+        <v>1</v>
+      </c>
+      <c r="H28" s="41">
+        <v>3</v>
+      </c>
+      <c r="I28" s="42" cm="1">
         <f t="array" ref="I28">IF(AND(ISNUMBER(G28),ISNUMBER(H28)),H28-G28,"")</f>
-      </c>
-      <c r="J28" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J28" t="s" s="43">
+        <v>161</v>
+      </c>
       <c r="K28" s="42"/>
       <c r="L28" s="44"/>
     </row>
@@ -4627,23 +4743,30 @@
         <v>68</v>
       </c>
       <c r="C29" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D29" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E29" t="s" s="40">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="F29" t="s" s="17">
-        <v>155</v>
-      </c>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" t="str" s="44" cm="1">
+        <v>163</v>
+      </c>
+      <c r="G29" s="41">
+        <v>1</v>
+      </c>
+      <c r="H29" s="41">
+        <v>3</v>
+      </c>
+      <c r="I29" s="42" cm="1">
         <f t="array" ref="I29">IF(AND(ISNUMBER(G29),ISNUMBER(H29)),H29-G29,"")</f>
-      </c>
-      <c r="J29" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J29" t="s" s="43">
+        <v>164</v>
+      </c>
       <c r="K29" s="42"/>
       <c r="L29" s="44"/>
     </row>
@@ -4655,23 +4778,30 @@
         <v>68</v>
       </c>
       <c r="C30" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D30" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E30" t="s" s="40">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="F30" t="s" s="17">
-        <v>157</v>
-      </c>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" t="str" s="44" cm="1">
+        <v>166</v>
+      </c>
+      <c r="G30" s="41">
+        <v>1</v>
+      </c>
+      <c r="H30" s="41">
+        <v>3</v>
+      </c>
+      <c r="I30" s="42" cm="1">
         <f t="array" ref="I30">IF(AND(ISNUMBER(G30),ISNUMBER(H30)),H30-G30,"")</f>
-      </c>
-      <c r="J30" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J30" t="s" s="43">
+        <v>167</v>
+      </c>
       <c r="K30" s="42"/>
       <c r="L30" s="44"/>
     </row>
@@ -4683,23 +4813,30 @@
         <v>68</v>
       </c>
       <c r="C31" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D31" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E31" t="s" s="40">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="F31" t="s" s="17">
-        <v>159</v>
-      </c>
-      <c r="G31" s="44"/>
-      <c r="H31" s="44"/>
-      <c r="I31" t="str" s="44" cm="1">
+        <v>169</v>
+      </c>
+      <c r="G31" s="41">
+        <v>1</v>
+      </c>
+      <c r="H31" s="41">
+        <v>3</v>
+      </c>
+      <c r="I31" s="42" cm="1">
         <f t="array" ref="I31">IF(AND(ISNUMBER(G31),ISNUMBER(H31)),H31-G31,"")</f>
-      </c>
-      <c r="J31" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J31" t="s" s="43">
+        <v>170</v>
+      </c>
       <c r="K31" s="42"/>
       <c r="L31" s="44"/>
     </row>
@@ -4711,2123 +4848,2130 @@
         <v>68</v>
       </c>
       <c r="C32" t="s" s="31">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D32" t="s" s="40">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E32" t="s" s="40">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="F32" t="s" s="17">
-        <v>161</v>
-      </c>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" t="str" s="44" cm="1">
+        <v>172</v>
+      </c>
+      <c r="G32" s="41">
+        <v>1</v>
+      </c>
+      <c r="H32" s="41">
+        <v>3</v>
+      </c>
+      <c r="I32" s="42" cm="1">
         <f t="array" ref="I32">IF(AND(ISNUMBER(G32),ISNUMBER(H32)),H32-G32,"")</f>
-      </c>
-      <c r="J32" s="46"/>
+        <v>2</v>
+      </c>
+      <c r="J32" t="s" s="43">
+        <v>173</v>
+      </c>
       <c r="K32" s="42"/>
       <c r="L32" s="44"/>
     </row>
     <row r="33" ht="36" customHeight="1">
-      <c r="A33" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B33" t="s" s="47">
-        <v>163</v>
+      <c r="A33" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C33" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D33" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E33" t="s" s="47">
-        <v>166</v>
+        <v>176</v>
+      </c>
+      <c r="D33" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E33" t="s" s="46">
+        <v>178</v>
       </c>
       <c r="F33" t="s" s="17">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="G33" s="44"/>
       <c r="H33" s="44"/>
       <c r="I33" t="str" s="44" cm="1">
         <f t="array" ref="I33">IF(AND(ISNUMBER(G33),ISNUMBER(H33)),H33-G33,"")</f>
       </c>
-      <c r="J33" s="46"/>
+      <c r="J33" s="47"/>
       <c r="K33" s="42"/>
       <c r="L33" s="44"/>
     </row>
     <row r="34" ht="36" customHeight="1">
-      <c r="A34" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B34" t="s" s="47">
-        <v>163</v>
+      <c r="A34" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B34" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C34" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D34" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E34" t="s" s="47">
-        <v>168</v>
+        <v>176</v>
+      </c>
+      <c r="D34" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E34" t="s" s="46">
+        <v>180</v>
       </c>
       <c r="F34" t="s" s="17">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="G34" s="44"/>
       <c r="H34" s="44"/>
       <c r="I34" t="str" s="44" cm="1">
         <f t="array" ref="I34">IF(AND(ISNUMBER(G34),ISNUMBER(H34)),H34-G34,"")</f>
       </c>
-      <c r="J34" s="46"/>
+      <c r="J34" s="47"/>
       <c r="K34" s="42"/>
       <c r="L34" s="44"/>
     </row>
     <row r="35" ht="36" customHeight="1">
-      <c r="A35" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B35" t="s" s="47">
-        <v>163</v>
+      <c r="A35" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B35" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C35" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D35" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E35" t="s" s="47">
-        <v>170</v>
+        <v>176</v>
+      </c>
+      <c r="D35" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E35" t="s" s="46">
+        <v>182</v>
       </c>
       <c r="F35" t="s" s="17">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="G35" s="44"/>
       <c r="H35" s="44"/>
       <c r="I35" t="str" s="44" cm="1">
         <f t="array" ref="I35">IF(AND(ISNUMBER(G35),ISNUMBER(H35)),H35-G35,"")</f>
       </c>
-      <c r="J35" s="46"/>
+      <c r="J35" s="47"/>
       <c r="K35" s="42"/>
       <c r="L35" s="44"/>
     </row>
     <row r="36" ht="36" customHeight="1">
-      <c r="A36" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B36" t="s" s="47">
-        <v>163</v>
+      <c r="A36" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B36" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C36" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D36" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E36" t="s" s="47">
-        <v>172</v>
+        <v>176</v>
+      </c>
+      <c r="D36" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E36" t="s" s="46">
+        <v>184</v>
       </c>
       <c r="F36" t="s" s="17">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="G36" s="44"/>
       <c r="H36" s="44"/>
       <c r="I36" t="str" s="44" cm="1">
         <f t="array" ref="I36">IF(AND(ISNUMBER(G36),ISNUMBER(H36)),H36-G36,"")</f>
       </c>
-      <c r="J36" s="46"/>
+      <c r="J36" s="47"/>
       <c r="K36" s="42"/>
       <c r="L36" s="44"/>
     </row>
     <row r="37" ht="36" customHeight="1">
-      <c r="A37" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B37" t="s" s="47">
-        <v>163</v>
+      <c r="A37" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B37" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C37" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D37" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E37" t="s" s="47">
-        <v>174</v>
+        <v>176</v>
+      </c>
+      <c r="D37" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E37" t="s" s="46">
+        <v>186</v>
       </c>
       <c r="F37" t="s" s="17">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="G37" s="44"/>
       <c r="H37" s="44"/>
       <c r="I37" t="str" s="44" cm="1">
         <f t="array" ref="I37">IF(AND(ISNUMBER(G37),ISNUMBER(H37)),H37-G37,"")</f>
       </c>
-      <c r="J37" s="46"/>
+      <c r="J37" s="47"/>
       <c r="K37" s="42"/>
       <c r="L37" s="44"/>
     </row>
     <row r="38" ht="36" customHeight="1">
-      <c r="A38" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B38" t="s" s="47">
-        <v>163</v>
+      <c r="A38" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B38" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C38" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D38" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E38" t="s" s="47">
         <v>176</v>
       </c>
+      <c r="D38" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E38" t="s" s="46">
+        <v>188</v>
+      </c>
       <c r="F38" t="s" s="17">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="G38" s="44"/>
       <c r="H38" s="44"/>
       <c r="I38" t="str" s="44" cm="1">
         <f t="array" ref="I38">IF(AND(ISNUMBER(G38),ISNUMBER(H38)),H38-G38,"")</f>
       </c>
-      <c r="J38" s="46"/>
+      <c r="J38" s="47"/>
       <c r="K38" s="42"/>
       <c r="L38" s="44"/>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B39" t="s" s="47">
-        <v>163</v>
+      <c r="A39" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B39" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C39" t="s" s="34">
-        <v>164</v>
-      </c>
-      <c r="D39" t="s" s="47">
-        <v>165</v>
-      </c>
-      <c r="E39" t="s" s="47">
-        <v>178</v>
+        <v>176</v>
+      </c>
+      <c r="D39" t="s" s="46">
+        <v>177</v>
+      </c>
+      <c r="E39" t="s" s="46">
+        <v>190</v>
       </c>
       <c r="F39" t="s" s="17">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="G39" s="44"/>
       <c r="H39" s="44"/>
       <c r="I39" t="str" s="44" cm="1">
         <f t="array" ref="I39">IF(AND(ISNUMBER(G39),ISNUMBER(H39)),H39-G39,"")</f>
       </c>
-      <c r="J39" s="46"/>
+      <c r="J39" s="47"/>
       <c r="K39" s="42"/>
       <c r="L39" s="44"/>
     </row>
     <row r="40" ht="36" customHeight="1">
-      <c r="A40" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B40" t="s" s="47">
-        <v>163</v>
+      <c r="A40" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B40" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C40" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D40" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E40" t="s" s="47">
-        <v>182</v>
+        <v>192</v>
+      </c>
+      <c r="D40" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E40" t="s" s="46">
+        <v>194</v>
       </c>
       <c r="F40" t="s" s="17">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="G40" s="44"/>
       <c r="H40" s="44"/>
       <c r="I40" t="str" s="44" cm="1">
         <f t="array" ref="I40">IF(AND(ISNUMBER(G40),ISNUMBER(H40)),H40-G40,"")</f>
       </c>
-      <c r="J40" s="46"/>
+      <c r="J40" s="47"/>
       <c r="K40" s="42"/>
       <c r="L40" s="44"/>
     </row>
     <row r="41" ht="36" customHeight="1">
-      <c r="A41" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B41" t="s" s="47">
-        <v>163</v>
+      <c r="A41" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B41" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C41" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D41" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E41" t="s" s="47">
-        <v>184</v>
+        <v>192</v>
+      </c>
+      <c r="D41" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E41" t="s" s="46">
+        <v>196</v>
       </c>
       <c r="F41" t="s" s="17">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="G41" s="44"/>
       <c r="H41" s="44"/>
       <c r="I41" t="str" s="44" cm="1">
         <f t="array" ref="I41">IF(AND(ISNUMBER(G41),ISNUMBER(H41)),H41-G41,"")</f>
       </c>
-      <c r="J41" s="46"/>
+      <c r="J41" s="47"/>
       <c r="K41" s="42"/>
       <c r="L41" s="44"/>
     </row>
     <row r="42" ht="36" customHeight="1">
-      <c r="A42" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B42" t="s" s="47">
-        <v>163</v>
+      <c r="A42" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B42" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C42" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D42" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E42" t="s" s="47">
-        <v>186</v>
+        <v>192</v>
+      </c>
+      <c r="D42" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E42" t="s" s="46">
+        <v>198</v>
       </c>
       <c r="F42" t="s" s="17">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="G42" s="44"/>
       <c r="H42" s="44"/>
       <c r="I42" t="str" s="44" cm="1">
         <f t="array" ref="I42">IF(AND(ISNUMBER(G42),ISNUMBER(H42)),H42-G42,"")</f>
       </c>
-      <c r="J42" s="46"/>
+      <c r="J42" s="47"/>
       <c r="K42" s="42"/>
       <c r="L42" s="44"/>
     </row>
     <row r="43" ht="36" customHeight="1">
-      <c r="A43" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B43" t="s" s="47">
-        <v>163</v>
+      <c r="A43" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B43" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C43" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D43" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E43" t="s" s="47">
-        <v>188</v>
+        <v>192</v>
+      </c>
+      <c r="D43" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E43" t="s" s="46">
+        <v>200</v>
       </c>
       <c r="F43" t="s" s="17">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="G43" s="44"/>
       <c r="H43" s="44"/>
       <c r="I43" t="str" s="44" cm="1">
         <f t="array" ref="I43">IF(AND(ISNUMBER(G43),ISNUMBER(H43)),H43-G43,"")</f>
       </c>
-      <c r="J43" s="46"/>
+      <c r="J43" s="47"/>
       <c r="K43" s="42"/>
       <c r="L43" s="44"/>
     </row>
     <row r="44" ht="36" customHeight="1">
-      <c r="A44" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B44" t="s" s="47">
-        <v>163</v>
+      <c r="A44" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B44" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C44" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D44" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E44" t="s" s="47">
-        <v>190</v>
+        <v>192</v>
+      </c>
+      <c r="D44" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E44" t="s" s="46">
+        <v>202</v>
       </c>
       <c r="F44" t="s" s="17">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="G44" s="44"/>
       <c r="H44" s="44"/>
       <c r="I44" t="str" s="44" cm="1">
         <f t="array" ref="I44">IF(AND(ISNUMBER(G44),ISNUMBER(H44)),H44-G44,"")</f>
       </c>
-      <c r="J44" s="46"/>
+      <c r="J44" s="47"/>
       <c r="K44" s="42"/>
       <c r="L44" s="44"/>
     </row>
     <row r="45" ht="36" customHeight="1">
-      <c r="A45" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B45" t="s" s="47">
-        <v>163</v>
+      <c r="A45" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B45" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C45" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D45" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E45" t="s" s="47">
         <v>192</v>
       </c>
+      <c r="D45" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E45" t="s" s="46">
+        <v>204</v>
+      </c>
       <c r="F45" t="s" s="17">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="G45" s="44"/>
       <c r="H45" s="44"/>
       <c r="I45" t="str" s="44" cm="1">
         <f t="array" ref="I45">IF(AND(ISNUMBER(G45),ISNUMBER(H45)),H45-G45,"")</f>
       </c>
-      <c r="J45" s="46"/>
+      <c r="J45" s="47"/>
       <c r="K45" s="42"/>
       <c r="L45" s="44"/>
     </row>
     <row r="46" ht="36" customHeight="1">
-      <c r="A46" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B46" t="s" s="47">
-        <v>163</v>
+      <c r="A46" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B46" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C46" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D46" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E46" t="s" s="47">
-        <v>194</v>
+        <v>192</v>
+      </c>
+      <c r="D46" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E46" t="s" s="46">
+        <v>206</v>
       </c>
       <c r="F46" t="s" s="17">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="G46" s="44"/>
       <c r="H46" s="44"/>
       <c r="I46" t="str" s="44" cm="1">
         <f t="array" ref="I46">IF(AND(ISNUMBER(G46),ISNUMBER(H46)),H46-G46,"")</f>
       </c>
-      <c r="J46" s="46"/>
+      <c r="J46" s="47"/>
       <c r="K46" s="42"/>
       <c r="L46" s="44"/>
     </row>
     <row r="47" ht="36" customHeight="1">
-      <c r="A47" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B47" t="s" s="47">
-        <v>163</v>
+      <c r="A47" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B47" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C47" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D47" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E47" t="s" s="47">
-        <v>196</v>
+        <v>192</v>
+      </c>
+      <c r="D47" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E47" t="s" s="46">
+        <v>208</v>
       </c>
       <c r="F47" t="s" s="17">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="G47" s="44"/>
       <c r="H47" s="44"/>
       <c r="I47" t="str" s="44" cm="1">
         <f t="array" ref="I47">IF(AND(ISNUMBER(G47),ISNUMBER(H47)),H47-G47,"")</f>
       </c>
-      <c r="J47" s="46"/>
+      <c r="J47" s="47"/>
       <c r="K47" s="42"/>
       <c r="L47" s="44"/>
     </row>
     <row r="48" ht="36" customHeight="1">
-      <c r="A48" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B48" t="s" s="47">
-        <v>163</v>
+      <c r="A48" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B48" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C48" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D48" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E48" t="s" s="47">
-        <v>198</v>
+        <v>192</v>
+      </c>
+      <c r="D48" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E48" t="s" s="46">
+        <v>210</v>
       </c>
       <c r="F48" t="s" s="17">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="G48" s="44"/>
       <c r="H48" s="44"/>
       <c r="I48" t="str" s="44" cm="1">
         <f t="array" ref="I48">IF(AND(ISNUMBER(G48),ISNUMBER(H48)),H48-G48,"")</f>
       </c>
-      <c r="J48" s="46"/>
+      <c r="J48" s="47"/>
       <c r="K48" s="42"/>
       <c r="L48" s="44"/>
     </row>
     <row r="49" ht="36" customHeight="1">
-      <c r="A49" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B49" t="s" s="47">
-        <v>163</v>
+      <c r="A49" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B49" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C49" t="s" s="34">
-        <v>180</v>
-      </c>
-      <c r="D49" t="s" s="47">
-        <v>181</v>
-      </c>
-      <c r="E49" t="s" s="47">
-        <v>200</v>
+        <v>192</v>
+      </c>
+      <c r="D49" t="s" s="46">
+        <v>193</v>
+      </c>
+      <c r="E49" t="s" s="46">
+        <v>212</v>
       </c>
       <c r="F49" t="s" s="17">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="G49" s="44"/>
       <c r="H49" s="44"/>
       <c r="I49" t="str" s="44" cm="1">
         <f t="array" ref="I49">IF(AND(ISNUMBER(G49),ISNUMBER(H49)),H49-G49,"")</f>
       </c>
-      <c r="J49" s="46"/>
+      <c r="J49" s="47"/>
       <c r="K49" s="42"/>
       <c r="L49" s="44"/>
     </row>
     <row r="50" ht="36" customHeight="1">
-      <c r="A50" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B50" t="s" s="47">
-        <v>163</v>
+      <c r="A50" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B50" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C50" t="s" s="34">
-        <v>202</v>
-      </c>
-      <c r="D50" t="s" s="47">
-        <v>203</v>
-      </c>
-      <c r="E50" t="s" s="47">
-        <v>204</v>
+        <v>214</v>
+      </c>
+      <c r="D50" t="s" s="46">
+        <v>215</v>
+      </c>
+      <c r="E50" t="s" s="46">
+        <v>216</v>
       </c>
       <c r="F50" t="s" s="17">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="G50" s="44"/>
       <c r="H50" s="44"/>
       <c r="I50" t="str" s="44" cm="1">
         <f t="array" ref="I50">IF(AND(ISNUMBER(G50),ISNUMBER(H50)),H50-G50,"")</f>
       </c>
-      <c r="J50" s="46"/>
+      <c r="J50" s="47"/>
       <c r="K50" s="42"/>
       <c r="L50" s="44"/>
     </row>
     <row r="51" ht="36" customHeight="1">
-      <c r="A51" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B51" t="s" s="47">
-        <v>163</v>
+      <c r="A51" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B51" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C51" t="s" s="34">
-        <v>202</v>
-      </c>
-      <c r="D51" t="s" s="47">
-        <v>203</v>
-      </c>
-      <c r="E51" t="s" s="47">
-        <v>206</v>
+        <v>214</v>
+      </c>
+      <c r="D51" t="s" s="46">
+        <v>215</v>
+      </c>
+      <c r="E51" t="s" s="46">
+        <v>218</v>
       </c>
       <c r="F51" t="s" s="17">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="G51" s="44"/>
       <c r="H51" s="44"/>
       <c r="I51" t="str" s="44" cm="1">
         <f t="array" ref="I51">IF(AND(ISNUMBER(G51),ISNUMBER(H51)),H51-G51,"")</f>
       </c>
-      <c r="J51" s="46"/>
+      <c r="J51" s="47"/>
       <c r="K51" s="42"/>
       <c r="L51" s="44"/>
     </row>
     <row r="52" ht="36" customHeight="1">
-      <c r="A52" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B52" t="s" s="47">
-        <v>163</v>
+      <c r="A52" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B52" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C52" t="s" s="34">
-        <v>202</v>
-      </c>
-      <c r="D52" t="s" s="47">
-        <v>203</v>
-      </c>
-      <c r="E52" t="s" s="47">
-        <v>208</v>
+        <v>214</v>
+      </c>
+      <c r="D52" t="s" s="46">
+        <v>215</v>
+      </c>
+      <c r="E52" t="s" s="46">
+        <v>220</v>
       </c>
       <c r="F52" t="s" s="17">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="G52" s="44"/>
       <c r="H52" s="44"/>
       <c r="I52" t="str" s="44" cm="1">
         <f t="array" ref="I52">IF(AND(ISNUMBER(G52),ISNUMBER(H52)),H52-G52,"")</f>
       </c>
-      <c r="J52" s="46"/>
+      <c r="J52" s="47"/>
       <c r="K52" s="42"/>
       <c r="L52" s="44"/>
     </row>
     <row r="53" ht="36" customHeight="1">
-      <c r="A53" t="s" s="47">
-        <v>162</v>
-      </c>
-      <c r="B53" t="s" s="47">
-        <v>163</v>
+      <c r="A53" t="s" s="46">
+        <v>174</v>
+      </c>
+      <c r="B53" t="s" s="46">
+        <v>175</v>
       </c>
       <c r="C53" t="s" s="34">
-        <v>202</v>
-      </c>
-      <c r="D53" t="s" s="47">
-        <v>203</v>
-      </c>
-      <c r="E53" t="s" s="47">
-        <v>210</v>
+        <v>214</v>
+      </c>
+      <c r="D53" t="s" s="46">
+        <v>215</v>
+      </c>
+      <c r="E53" t="s" s="46">
+        <v>222</v>
       </c>
       <c r="F53" t="s" s="17">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="G53" s="44"/>
       <c r="H53" s="44"/>
       <c r="I53" t="str" s="44" cm="1">
         <f t="array" ref="I53">IF(AND(ISNUMBER(G53),ISNUMBER(H53)),H53-G53,"")</f>
       </c>
-      <c r="J53" s="46"/>
+      <c r="J53" s="47"/>
       <c r="K53" s="42"/>
       <c r="L53" s="44"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B54" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C54" t="s" s="29">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D54" t="s" s="48">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E54" t="s" s="48">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="F54" t="s" s="17">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="G54" s="44"/>
       <c r="H54" s="44"/>
       <c r="I54" t="str" s="44" cm="1">
         <f t="array" ref="I54">IF(AND(ISNUMBER(G54),ISNUMBER(H54)),H54-G54,"")</f>
       </c>
-      <c r="J54" s="46"/>
+      <c r="J54" s="47"/>
       <c r="K54" s="42"/>
       <c r="L54" s="44"/>
     </row>
     <row r="55" ht="36" customHeight="1">
       <c r="A55" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B55" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C55" t="s" s="29">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D55" t="s" s="48">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E55" t="s" s="48">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="F55" t="s" s="17">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="G55" s="44"/>
       <c r="H55" s="44"/>
       <c r="I55" t="str" s="44" cm="1">
         <f t="array" ref="I55">IF(AND(ISNUMBER(G55),ISNUMBER(H55)),H55-G55,"")</f>
       </c>
-      <c r="J55" s="46"/>
+      <c r="J55" s="47"/>
       <c r="K55" s="42"/>
       <c r="L55" s="44"/>
     </row>
     <row r="56" ht="36" customHeight="1">
       <c r="A56" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B56" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C56" t="s" s="29">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D56" t="s" s="48">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E56" t="s" s="48">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="F56" t="s" s="17">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="G56" s="44"/>
       <c r="H56" s="44"/>
       <c r="I56" t="str" s="44" cm="1">
         <f t="array" ref="I56">IF(AND(ISNUMBER(G56),ISNUMBER(H56)),H56-G56,"")</f>
       </c>
-      <c r="J56" s="46"/>
+      <c r="J56" s="47"/>
       <c r="K56" s="42"/>
       <c r="L56" s="44"/>
     </row>
     <row r="57" ht="36" customHeight="1">
       <c r="A57" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B57" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C57" t="s" s="29">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D57" t="s" s="48">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E57" t="s" s="48">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="F57" t="s" s="17">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="G57" s="44"/>
       <c r="H57" s="44"/>
       <c r="I57" t="str" s="44" cm="1">
         <f t="array" ref="I57">IF(AND(ISNUMBER(G57),ISNUMBER(H57)),H57-G57,"")</f>
       </c>
-      <c r="J57" s="46"/>
+      <c r="J57" s="47"/>
       <c r="K57" s="42"/>
       <c r="L57" s="44"/>
     </row>
     <row r="58" ht="36" customHeight="1">
       <c r="A58" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B58" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C58" t="s" s="29">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D58" t="s" s="48">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E58" t="s" s="48">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="F58" t="s" s="17">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="G58" s="44"/>
       <c r="H58" s="44"/>
       <c r="I58" t="str" s="44" cm="1">
         <f t="array" ref="I58">IF(AND(ISNUMBER(G58),ISNUMBER(H58)),H58-G58,"")</f>
       </c>
-      <c r="J58" s="46"/>
+      <c r="J58" s="47"/>
       <c r="K58" s="42"/>
       <c r="L58" s="44"/>
     </row>
     <row r="59" ht="36" customHeight="1">
       <c r="A59" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B59" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C59" t="s" s="29">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D59" t="s" s="48">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E59" t="s" s="48">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="F59" t="s" s="17">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="G59" s="44"/>
       <c r="H59" s="44"/>
       <c r="I59" t="str" s="44" cm="1">
         <f t="array" ref="I59">IF(AND(ISNUMBER(G59),ISNUMBER(H59)),H59-G59,"")</f>
       </c>
-      <c r="J59" s="46"/>
+      <c r="J59" s="47"/>
       <c r="K59" s="42"/>
       <c r="L59" s="44"/>
     </row>
     <row r="60" ht="36" customHeight="1">
       <c r="A60" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B60" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C60" t="s" s="29">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="D60" t="s" s="48">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="E60" t="s" s="48">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="F60" t="s" s="17">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="G60" s="44"/>
       <c r="H60" s="44"/>
       <c r="I60" t="str" s="44" cm="1">
         <f t="array" ref="I60">IF(AND(ISNUMBER(G60),ISNUMBER(H60)),H60-G60,"")</f>
       </c>
-      <c r="J60" s="46"/>
+      <c r="J60" s="47"/>
       <c r="K60" s="42"/>
       <c r="L60" s="44"/>
     </row>
     <row r="61" ht="36" customHeight="1">
       <c r="A61" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B61" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C61" t="s" s="29">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="D61" t="s" s="48">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="E61" t="s" s="48">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="F61" t="s" s="17">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="G61" s="44"/>
       <c r="H61" s="44"/>
       <c r="I61" t="str" s="44" cm="1">
         <f t="array" ref="I61">IF(AND(ISNUMBER(G61),ISNUMBER(H61)),H61-G61,"")</f>
       </c>
-      <c r="J61" s="46"/>
+      <c r="J61" s="47"/>
       <c r="K61" s="42"/>
       <c r="L61" s="44"/>
     </row>
     <row r="62" ht="36" customHeight="1">
       <c r="A62" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B62" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C62" t="s" s="29">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D62" t="s" s="48">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E62" t="s" s="48">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="F62" t="s" s="17">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="G62" s="44"/>
       <c r="H62" s="44"/>
       <c r="I62" t="str" s="44" cm="1">
         <f t="array" ref="I62">IF(AND(ISNUMBER(G62),ISNUMBER(H62)),H62-G62,"")</f>
       </c>
-      <c r="J62" s="46"/>
+      <c r="J62" s="47"/>
       <c r="K62" s="42"/>
       <c r="L62" s="44"/>
     </row>
     <row r="63" ht="36" customHeight="1">
       <c r="A63" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B63" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C63" t="s" s="29">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D63" t="s" s="48">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E63" t="s" s="48">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="F63" t="s" s="17">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="G63" s="44"/>
       <c r="H63" s="44"/>
       <c r="I63" t="str" s="44" cm="1">
         <f t="array" ref="I63">IF(AND(ISNUMBER(G63),ISNUMBER(H63)),H63-G63,"")</f>
       </c>
-      <c r="J63" s="46"/>
+      <c r="J63" s="47"/>
       <c r="K63" s="42"/>
       <c r="L63" s="44"/>
     </row>
     <row r="64" ht="36" customHeight="1">
       <c r="A64" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B64" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C64" t="s" s="29">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D64" t="s" s="48">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E64" t="s" s="48">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="F64" t="s" s="17">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="G64" s="44"/>
       <c r="H64" s="44"/>
       <c r="I64" t="str" s="44" cm="1">
         <f t="array" ref="I64">IF(AND(ISNUMBER(G64),ISNUMBER(H64)),H64-G64,"")</f>
       </c>
-      <c r="J64" s="46"/>
+      <c r="J64" s="47"/>
       <c r="K64" s="42"/>
       <c r="L64" s="44"/>
     </row>
     <row r="65" ht="36" customHeight="1">
       <c r="A65" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B65" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C65" t="s" s="29">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D65" t="s" s="48">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E65" t="s" s="48">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="F65" t="s" s="17">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="G65" s="44"/>
       <c r="H65" s="44"/>
       <c r="I65" t="str" s="44" cm="1">
         <f t="array" ref="I65">IF(AND(ISNUMBER(G65),ISNUMBER(H65)),H65-G65,"")</f>
       </c>
-      <c r="J65" s="46"/>
+      <c r="J65" s="47"/>
       <c r="K65" s="42"/>
       <c r="L65" s="44"/>
     </row>
     <row r="66" ht="36" customHeight="1">
       <c r="A66" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B66" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C66" t="s" s="29">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D66" t="s" s="48">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E66" t="s" s="48">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="F66" t="s" s="17">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="G66" s="44"/>
       <c r="H66" s="44"/>
       <c r="I66" t="str" s="44" cm="1">
         <f t="array" ref="I66">IF(AND(ISNUMBER(G66),ISNUMBER(H66)),H66-G66,"")</f>
       </c>
-      <c r="J66" s="46"/>
+      <c r="J66" s="47"/>
       <c r="K66" s="42"/>
       <c r="L66" s="44"/>
     </row>
     <row r="67" ht="36" customHeight="1">
       <c r="A67" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B67" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C67" t="s" s="29">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D67" t="s" s="48">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E67" t="s" s="48">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="F67" t="s" s="17">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="G67" s="44"/>
       <c r="H67" s="44"/>
       <c r="I67" t="str" s="44" cm="1">
         <f t="array" ref="I67">IF(AND(ISNUMBER(G67),ISNUMBER(H67)),H67-G67,"")</f>
       </c>
-      <c r="J67" s="46"/>
+      <c r="J67" s="47"/>
       <c r="K67" s="42"/>
       <c r="L67" s="44"/>
     </row>
     <row r="68" ht="36" customHeight="1">
       <c r="A68" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B68" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C68" t="s" s="29">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D68" t="s" s="48">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E68" t="s" s="48">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="F68" t="s" s="17">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="G68" s="44"/>
       <c r="H68" s="44"/>
       <c r="I68" t="str" s="44" cm="1">
         <f t="array" ref="I68">IF(AND(ISNUMBER(G68),ISNUMBER(H68)),H68-G68,"")</f>
       </c>
-      <c r="J68" s="46"/>
+      <c r="J68" s="47"/>
       <c r="K68" s="42"/>
       <c r="L68" s="44"/>
     </row>
     <row r="69" ht="36" customHeight="1">
       <c r="A69" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B69" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C69" t="s" s="29">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D69" t="s" s="48">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E69" t="s" s="48">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F69" t="s" s="17">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="G69" s="44"/>
       <c r="H69" s="44"/>
       <c r="I69" t="str" s="44" cm="1">
         <f t="array" ref="I69">IF(AND(ISNUMBER(G69),ISNUMBER(H69)),H69-G69,"")</f>
       </c>
-      <c r="J69" s="46"/>
+      <c r="J69" s="47"/>
       <c r="K69" s="42"/>
       <c r="L69" s="44"/>
     </row>
     <row r="70" ht="36" customHeight="1">
       <c r="A70" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B70" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C70" t="s" s="29">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D70" t="s" s="48">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E70" t="s" s="48">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F70" t="s" s="17">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="G70" s="44"/>
       <c r="H70" s="44"/>
       <c r="I70" t="str" s="44" cm="1">
         <f t="array" ref="I70">IF(AND(ISNUMBER(G70),ISNUMBER(H70)),H70-G70,"")</f>
       </c>
-      <c r="J70" s="46"/>
+      <c r="J70" s="47"/>
       <c r="K70" s="42"/>
       <c r="L70" s="44"/>
     </row>
     <row r="71" ht="36" customHeight="1">
       <c r="A71" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B71" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C71" t="s" s="29">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D71" t="s" s="48">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E71" t="s" s="48">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F71" t="s" s="17">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="G71" s="44"/>
       <c r="H71" s="44"/>
       <c r="I71" t="str" s="44" cm="1">
         <f t="array" ref="I71">IF(AND(ISNUMBER(G71),ISNUMBER(H71)),H71-G71,"")</f>
       </c>
-      <c r="J71" s="46"/>
+      <c r="J71" s="47"/>
       <c r="K71" s="42"/>
       <c r="L71" s="44"/>
     </row>
     <row r="72" ht="36" customHeight="1">
       <c r="A72" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B72" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C72" t="s" s="29">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D72" t="s" s="48">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E72" t="s" s="48">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="F72" t="s" s="17">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="G72" s="44"/>
       <c r="H72" s="44"/>
       <c r="I72" t="str" s="44" cm="1">
         <f t="array" ref="I72">IF(AND(ISNUMBER(G72),ISNUMBER(H72)),H72-G72,"")</f>
       </c>
-      <c r="J72" s="46"/>
+      <c r="J72" s="47"/>
       <c r="K72" s="42"/>
       <c r="L72" s="44"/>
     </row>
     <row r="73" ht="36" customHeight="1">
       <c r="A73" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B73" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C73" t="s" s="29">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D73" t="s" s="48">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E73" t="s" s="48">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="F73" t="s" s="17">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="G73" s="44"/>
       <c r="H73" s="44"/>
       <c r="I73" t="str" s="44" cm="1">
         <f t="array" ref="I73">IF(AND(ISNUMBER(G73),ISNUMBER(H73)),H73-G73,"")</f>
       </c>
-      <c r="J73" s="46"/>
+      <c r="J73" s="47"/>
       <c r="K73" s="42"/>
       <c r="L73" s="44"/>
     </row>
     <row r="74" ht="36" customHeight="1">
       <c r="A74" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B74" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C74" t="s" s="29">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D74" t="s" s="48">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E74" t="s" s="48">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="F74" t="s" s="17">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="G74" s="44"/>
       <c r="H74" s="44"/>
       <c r="I74" t="str" s="44" cm="1">
         <f t="array" ref="I74">IF(AND(ISNUMBER(G74),ISNUMBER(H74)),H74-G74,"")</f>
       </c>
-      <c r="J74" s="46"/>
+      <c r="J74" s="47"/>
       <c r="K74" s="42"/>
       <c r="L74" s="44"/>
     </row>
     <row r="75" ht="36" customHeight="1">
       <c r="A75" t="s" s="48">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B75" t="s" s="48">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C75" t="s" s="29">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D75" t="s" s="48">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E75" t="s" s="48">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="F75" t="s" s="17">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="G75" s="44"/>
       <c r="H75" s="44"/>
       <c r="I75" t="str" s="44" cm="1">
         <f t="array" ref="I75">IF(AND(ISNUMBER(G75),ISNUMBER(H75)),H75-G75,"")</f>
       </c>
-      <c r="J75" s="46"/>
+      <c r="J75" s="47"/>
       <c r="K75" s="42"/>
       <c r="L75" s="44"/>
     </row>
     <row r="76" ht="36" customHeight="1">
       <c r="A76" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B76" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C76" t="s" s="26">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D76" t="s" s="49">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="E76" t="s" s="49">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="F76" t="s" s="17">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="G76" s="44"/>
       <c r="H76" s="44"/>
       <c r="I76" t="str" s="44" cm="1">
         <f t="array" ref="I76">IF(AND(ISNUMBER(G76),ISNUMBER(H76)),H76-G76,"")</f>
       </c>
-      <c r="J76" s="46"/>
+      <c r="J76" s="47"/>
       <c r="K76" s="42"/>
       <c r="L76" s="44"/>
     </row>
     <row r="77" ht="36" customHeight="1">
       <c r="A77" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B77" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C77" t="s" s="26">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D77" t="s" s="49">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="E77" t="s" s="49">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="F77" t="s" s="17">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="G77" s="44"/>
       <c r="H77" s="44"/>
       <c r="I77" t="str" s="44" cm="1">
         <f t="array" ref="I77">IF(AND(ISNUMBER(G77),ISNUMBER(H77)),H77-G77,"")</f>
       </c>
-      <c r="J77" s="46"/>
+      <c r="J77" s="47"/>
       <c r="K77" s="42"/>
       <c r="L77" s="44"/>
     </row>
     <row r="78" ht="36" customHeight="1">
       <c r="A78" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B78" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C78" t="s" s="26">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D78" t="s" s="49">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="E78" t="s" s="49">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="F78" t="s" s="17">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="G78" s="44"/>
       <c r="H78" s="44"/>
       <c r="I78" t="str" s="44" cm="1">
         <f t="array" ref="I78">IF(AND(ISNUMBER(G78),ISNUMBER(H78)),H78-G78,"")</f>
       </c>
-      <c r="J78" s="46"/>
+      <c r="J78" s="47"/>
       <c r="K78" s="42"/>
       <c r="L78" s="44"/>
     </row>
     <row r="79" ht="36" customHeight="1">
       <c r="A79" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B79" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C79" t="s" s="26">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D79" t="s" s="49">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="E79" t="s" s="49">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="F79" t="s" s="17">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="G79" s="44"/>
       <c r="H79" s="44"/>
       <c r="I79" t="str" s="44" cm="1">
         <f t="array" ref="I79">IF(AND(ISNUMBER(G79),ISNUMBER(H79)),H79-G79,"")</f>
       </c>
-      <c r="J79" s="46"/>
+      <c r="J79" s="47"/>
       <c r="K79" s="42"/>
       <c r="L79" s="44"/>
     </row>
     <row r="80" ht="36" customHeight="1">
       <c r="A80" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B80" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C80" t="s" s="26">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="D80" t="s" s="49">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="E80" t="s" s="49">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="F80" t="s" s="17">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="G80" s="44"/>
       <c r="H80" s="44"/>
       <c r="I80" t="str" s="44" cm="1">
         <f t="array" ref="I80">IF(AND(ISNUMBER(G80),ISNUMBER(H80)),H80-G80,"")</f>
       </c>
-      <c r="J80" s="46"/>
+      <c r="J80" s="47"/>
       <c r="K80" s="42"/>
       <c r="L80" s="44"/>
     </row>
     <row r="81" ht="36" customHeight="1">
       <c r="A81" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B81" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C81" t="s" s="26">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D81" t="s" s="49">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E81" t="s" s="49">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="F81" t="s" s="17">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="G81" s="44"/>
       <c r="H81" s="44"/>
       <c r="I81" t="str" s="44" cm="1">
         <f t="array" ref="I81">IF(AND(ISNUMBER(G81),ISNUMBER(H81)),H81-G81,"")</f>
       </c>
-      <c r="J81" s="46"/>
+      <c r="J81" s="47"/>
       <c r="K81" s="42"/>
       <c r="L81" s="44"/>
     </row>
     <row r="82" ht="36" customHeight="1">
       <c r="A82" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B82" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C82" t="s" s="26">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D82" t="s" s="49">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E82" t="s" s="49">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="F82" t="s" s="17">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="G82" s="44"/>
       <c r="H82" s="44"/>
       <c r="I82" t="str" s="44" cm="1">
         <f t="array" ref="I82">IF(AND(ISNUMBER(G82),ISNUMBER(H82)),H82-G82,"")</f>
       </c>
-      <c r="J82" s="46"/>
+      <c r="J82" s="47"/>
       <c r="K82" s="42"/>
       <c r="L82" s="44"/>
     </row>
     <row r="83" ht="36" customHeight="1">
       <c r="A83" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B83" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C83" t="s" s="26">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D83" t="s" s="49">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E83" t="s" s="49">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="F83" t="s" s="17">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="G83" s="44"/>
       <c r="H83" s="44"/>
       <c r="I83" t="str" s="44" cm="1">
         <f t="array" ref="I83">IF(AND(ISNUMBER(G83),ISNUMBER(H83)),H83-G83,"")</f>
       </c>
-      <c r="J83" s="46"/>
+      <c r="J83" s="47"/>
       <c r="K83" s="42"/>
       <c r="L83" s="44"/>
     </row>
     <row r="84" ht="36" customHeight="1">
       <c r="A84" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B84" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C84" t="s" s="26">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D84" t="s" s="49">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E84" t="s" s="49">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="F84" t="s" s="17">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="G84" s="44"/>
       <c r="H84" s="44"/>
       <c r="I84" t="str" s="44" cm="1">
         <f t="array" ref="I84">IF(AND(ISNUMBER(G84),ISNUMBER(H84)),H84-G84,"")</f>
       </c>
-      <c r="J84" s="46"/>
+      <c r="J84" s="47"/>
       <c r="K84" s="42"/>
       <c r="L84" s="44"/>
     </row>
     <row r="85" ht="36" customHeight="1">
       <c r="A85" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B85" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C85" t="s" s="26">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D85" t="s" s="49">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E85" t="s" s="49">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="F85" t="s" s="17">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="G85" s="44"/>
       <c r="H85" s="44"/>
       <c r="I85" t="str" s="44" cm="1">
         <f t="array" ref="I85">IF(AND(ISNUMBER(G85),ISNUMBER(H85)),H85-G85,"")</f>
       </c>
-      <c r="J85" s="46"/>
+      <c r="J85" s="47"/>
       <c r="K85" s="42"/>
       <c r="L85" s="44"/>
     </row>
     <row r="86" ht="36" customHeight="1">
       <c r="A86" t="s" s="49">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B86" t="s" s="49">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C86" t="s" s="26">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="D86" t="s" s="49">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E86" t="s" s="49">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="F86" t="s" s="17">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="G86" s="44"/>
       <c r="H86" s="44"/>
       <c r="I86" t="str" s="44" cm="1">
         <f t="array" ref="I86">IF(AND(ISNUMBER(G86),ISNUMBER(H86)),H86-G86,"")</f>
       </c>
-      <c r="J86" s="46"/>
+      <c r="J86" s="47"/>
       <c r="K86" s="42"/>
       <c r="L86" s="44"/>
     </row>
     <row r="87" ht="36" customHeight="1">
       <c r="A87" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B87" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C87" t="s" s="51">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="D87" t="s" s="50">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="E87" t="s" s="50">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="F87" t="s" s="17">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="G87" s="44"/>
       <c r="H87" s="44"/>
       <c r="I87" t="str" s="44" cm="1">
         <f t="array" ref="I87">IF(AND(ISNUMBER(G87),ISNUMBER(H87)),H87-G87,"")</f>
       </c>
-      <c r="J87" s="46"/>
+      <c r="J87" s="47"/>
       <c r="K87" s="42"/>
       <c r="L87" s="44"/>
     </row>
     <row r="88" ht="36" customHeight="1">
       <c r="A88" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B88" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C88" t="s" s="51">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="D88" t="s" s="50">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="E88" t="s" s="50">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="F88" t="s" s="17">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="G88" s="44"/>
       <c r="H88" s="44"/>
       <c r="I88" t="str" s="44" cm="1">
         <f t="array" ref="I88">IF(AND(ISNUMBER(G88),ISNUMBER(H88)),H88-G88,"")</f>
       </c>
-      <c r="J88" s="46"/>
+      <c r="J88" s="47"/>
       <c r="K88" s="42"/>
       <c r="L88" s="44"/>
     </row>
     <row r="89" ht="36" customHeight="1">
       <c r="A89" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B89" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C89" t="s" s="51">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="D89" t="s" s="50">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="E89" t="s" s="50">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="F89" t="s" s="17">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="G89" s="44"/>
       <c r="H89" s="44"/>
       <c r="I89" t="str" s="44" cm="1">
         <f t="array" ref="I89">IF(AND(ISNUMBER(G89),ISNUMBER(H89)),H89-G89,"")</f>
       </c>
-      <c r="J89" s="46"/>
+      <c r="J89" s="47"/>
       <c r="K89" s="42"/>
       <c r="L89" s="44"/>
     </row>
     <row r="90" ht="36" customHeight="1">
       <c r="A90" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B90" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C90" t="s" s="51">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="D90" t="s" s="50">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="E90" t="s" s="50">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="F90" t="s" s="17">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="G90" s="44"/>
       <c r="H90" s="44"/>
       <c r="I90" t="str" s="44" cm="1">
         <f t="array" ref="I90">IF(AND(ISNUMBER(G90),ISNUMBER(H90)),H90-G90,"")</f>
       </c>
-      <c r="J90" s="46"/>
+      <c r="J90" s="47"/>
       <c r="K90" s="42"/>
       <c r="L90" s="44"/>
     </row>
     <row r="91" ht="36" customHeight="1">
       <c r="A91" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B91" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C91" t="s" s="51">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="D91" t="s" s="50">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="E91" t="s" s="50">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="F91" t="s" s="17">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="G91" s="44"/>
       <c r="H91" s="44"/>
       <c r="I91" t="str" s="44" cm="1">
         <f t="array" ref="I91">IF(AND(ISNUMBER(G91),ISNUMBER(H91)),H91-G91,"")</f>
       </c>
-      <c r="J91" s="46"/>
+      <c r="J91" s="47"/>
       <c r="K91" s="42"/>
       <c r="L91" s="44"/>
     </row>
     <row r="92" ht="36" customHeight="1">
       <c r="A92" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B92" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C92" t="s" s="51">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="D92" t="s" s="50">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="E92" t="s" s="50">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="F92" t="s" s="17">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="G92" s="44"/>
       <c r="H92" s="44"/>
       <c r="I92" t="str" s="44" cm="1">
         <f t="array" ref="I92">IF(AND(ISNUMBER(G92),ISNUMBER(H92)),H92-G92,"")</f>
       </c>
-      <c r="J92" s="46"/>
+      <c r="J92" s="47"/>
       <c r="K92" s="42"/>
       <c r="L92" s="44"/>
     </row>
     <row r="93" ht="36" customHeight="1">
       <c r="A93" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B93" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C93" t="s" s="51">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="D93" t="s" s="50">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="E93" t="s" s="50">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="F93" t="s" s="17">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="G93" s="44"/>
       <c r="H93" s="44"/>
       <c r="I93" t="str" s="44" cm="1">
         <f t="array" ref="I93">IF(AND(ISNUMBER(G93),ISNUMBER(H93)),H93-G93,"")</f>
       </c>
-      <c r="J93" s="46"/>
+      <c r="J93" s="47"/>
       <c r="K93" s="42"/>
       <c r="L93" s="44"/>
     </row>
     <row r="94" ht="36" customHeight="1">
       <c r="A94" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B94" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C94" t="s" s="51">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="D94" t="s" s="50">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="E94" t="s" s="50">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="F94" t="s" s="17">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="G94" s="44"/>
       <c r="H94" s="44"/>
       <c r="I94" t="str" s="44" cm="1">
         <f t="array" ref="I94">IF(AND(ISNUMBER(G94),ISNUMBER(H94)),H94-G94,"")</f>
       </c>
-      <c r="J94" s="46"/>
+      <c r="J94" s="47"/>
       <c r="K94" s="42"/>
       <c r="L94" s="44"/>
     </row>
     <row r="95" ht="36" customHeight="1">
       <c r="A95" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B95" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C95" t="s" s="51">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="D95" t="s" s="50">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="E95" t="s" s="50">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="F95" t="s" s="17">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="G95" s="44"/>
       <c r="H95" s="44"/>
       <c r="I95" t="str" s="44" cm="1">
         <f t="array" ref="I95">IF(AND(ISNUMBER(G95),ISNUMBER(H95)),H95-G95,"")</f>
       </c>
-      <c r="J95" s="46"/>
+      <c r="J95" s="47"/>
       <c r="K95" s="42"/>
       <c r="L95" s="44"/>
     </row>
     <row r="96" ht="36" customHeight="1">
       <c r="A96" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B96" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C96" t="s" s="51">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="D96" t="s" s="50">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="E96" t="s" s="50">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="F96" t="s" s="17">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="G96" s="44"/>
       <c r="H96" s="44"/>
       <c r="I96" t="str" s="44" cm="1">
         <f t="array" ref="I96">IF(AND(ISNUMBER(G96),ISNUMBER(H96)),H96-G96,"")</f>
       </c>
-      <c r="J96" s="46"/>
+      <c r="J96" s="47"/>
       <c r="K96" s="42"/>
       <c r="L96" s="44"/>
     </row>
     <row r="97" ht="36" customHeight="1">
       <c r="A97" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B97" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C97" t="s" s="51">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="D97" t="s" s="50">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="E97" t="s" s="50">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="F97" t="s" s="17">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="G97" s="44"/>
       <c r="H97" s="44"/>
       <c r="I97" t="str" s="44" cm="1">
         <f t="array" ref="I97">IF(AND(ISNUMBER(G97),ISNUMBER(H97)),H97-G97,"")</f>
       </c>
-      <c r="J97" s="46"/>
+      <c r="J97" s="47"/>
       <c r="K97" s="42"/>
       <c r="L97" s="44"/>
     </row>
     <row r="98" ht="36" customHeight="1">
       <c r="A98" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B98" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C98" t="s" s="51">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="D98" t="s" s="50">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="E98" t="s" s="50">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="F98" t="s" s="17">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="G98" s="44"/>
       <c r="H98" s="44"/>
       <c r="I98" t="str" s="44" cm="1">
         <f t="array" ref="I98">IF(AND(ISNUMBER(G98),ISNUMBER(H98)),H98-G98,"")</f>
       </c>
-      <c r="J98" s="46"/>
+      <c r="J98" s="47"/>
       <c r="K98" s="42"/>
       <c r="L98" s="44"/>
     </row>
     <row r="99" ht="36" customHeight="1">
       <c r="A99" t="s" s="50">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B99" t="s" s="50">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C99" t="s" s="51">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="D99" t="s" s="50">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="E99" t="s" s="50">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="F99" t="s" s="17">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="G99" s="44"/>
       <c r="H99" s="44"/>
       <c r="I99" t="str" s="44" cm="1">
         <f t="array" ref="I99">IF(AND(ISNUMBER(G99),ISNUMBER(H99)),H99-G99,"")</f>
       </c>
-      <c r="J99" s="46"/>
+      <c r="J99" s="47"/>
       <c r="K99" s="42"/>
       <c r="L99" s="44"/>
     </row>
     <row r="100" ht="36" customHeight="1">
       <c r="A100" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B100" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C100" t="s" s="53">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D100" t="s" s="52">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E100" t="s" s="52">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="F100" t="s" s="17">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="G100" s="44"/>
       <c r="H100" s="44"/>
       <c r="I100" t="str" s="44" cm="1">
         <f t="array" ref="I100">IF(AND(ISNUMBER(G100),ISNUMBER(H100)),H100-G100,"")</f>
       </c>
-      <c r="J100" s="46"/>
+      <c r="J100" s="47"/>
       <c r="K100" s="42"/>
       <c r="L100" s="44"/>
     </row>
     <row r="101" ht="36" customHeight="1">
       <c r="A101" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B101" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C101" t="s" s="53">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D101" t="s" s="52">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E101" t="s" s="52">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="F101" t="s" s="17">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="G101" s="44"/>
       <c r="H101" s="44"/>
       <c r="I101" t="str" s="44" cm="1">
         <f t="array" ref="I101">IF(AND(ISNUMBER(G101),ISNUMBER(H101)),H101-G101,"")</f>
       </c>
-      <c r="J101" s="46"/>
+      <c r="J101" s="47"/>
       <c r="K101" s="42"/>
       <c r="L101" s="44"/>
     </row>
     <row r="102" ht="36" customHeight="1">
       <c r="A102" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B102" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C102" t="s" s="53">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D102" t="s" s="52">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E102" t="s" s="52">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="F102" t="s" s="17">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="G102" s="44"/>
       <c r="H102" s="44"/>
       <c r="I102" t="str" s="44" cm="1">
         <f t="array" ref="I102">IF(AND(ISNUMBER(G102),ISNUMBER(H102)),H102-G102,"")</f>
       </c>
-      <c r="J102" s="46"/>
+      <c r="J102" s="47"/>
       <c r="K102" s="42"/>
       <c r="L102" s="44"/>
     </row>
     <row r="103" ht="36" customHeight="1">
       <c r="A103" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B103" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C103" t="s" s="53">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D103" t="s" s="52">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E103" t="s" s="52">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="F103" t="s" s="17">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="G103" s="44"/>
       <c r="H103" s="44"/>
       <c r="I103" t="str" s="44" cm="1">
         <f t="array" ref="I103">IF(AND(ISNUMBER(G103),ISNUMBER(H103)),H103-G103,"")</f>
       </c>
-      <c r="J103" s="46"/>
+      <c r="J103" s="47"/>
       <c r="K103" s="42"/>
       <c r="L103" s="44"/>
     </row>
     <row r="104" ht="36" customHeight="1">
       <c r="A104" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B104" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C104" t="s" s="53">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D104" t="s" s="52">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E104" t="s" s="52">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="F104" t="s" s="17">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="G104" s="44"/>
       <c r="H104" s="44"/>
       <c r="I104" t="str" s="44" cm="1">
         <f t="array" ref="I104">IF(AND(ISNUMBER(G104),ISNUMBER(H104)),H104-G104,"")</f>
       </c>
-      <c r="J104" s="46"/>
+      <c r="J104" s="47"/>
       <c r="K104" s="42"/>
       <c r="L104" s="44"/>
     </row>
     <row r="105" ht="36" customHeight="1">
       <c r="A105" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B105" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C105" t="s" s="53">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D105" t="s" s="52">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E105" t="s" s="52">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="F105" t="s" s="17">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="G105" s="44"/>
       <c r="H105" s="44"/>
       <c r="I105" t="str" s="44" cm="1">
         <f t="array" ref="I105">IF(AND(ISNUMBER(G105),ISNUMBER(H105)),H105-G105,"")</f>
       </c>
-      <c r="J105" s="46"/>
+      <c r="J105" s="47"/>
       <c r="K105" s="42"/>
       <c r="L105" s="44"/>
     </row>
     <row r="106" ht="36" customHeight="1">
       <c r="A106" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B106" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C106" t="s" s="53">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="D106" t="s" s="52">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="E106" t="s" s="52">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="F106" t="s" s="17">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="G106" s="44"/>
       <c r="H106" s="44"/>
       <c r="I106" t="str" s="44" cm="1">
         <f t="array" ref="I106">IF(AND(ISNUMBER(G106),ISNUMBER(H106)),H106-G106,"")</f>
       </c>
-      <c r="J106" s="46"/>
+      <c r="J106" s="47"/>
       <c r="K106" s="42"/>
       <c r="L106" s="44"/>
     </row>
     <row r="107" ht="36" customHeight="1">
       <c r="A107" t="s" s="52">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B107" t="s" s="52">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C107" t="s" s="53">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="D107" t="s" s="52">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="E107" t="s" s="52">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="F107" t="s" s="17">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="G107" s="44"/>
       <c r="H107" s="44"/>
       <c r="I107" t="str" s="44" cm="1">
         <f t="array" ref="I107">IF(AND(ISNUMBER(G107),ISNUMBER(H107)),H107-G107,"")</f>
       </c>
-      <c r="J107" s="46"/>
+      <c r="J107" s="47"/>
       <c r="K107" s="42"/>
       <c r="L107" s="44"/>
     </row>
@@ -6870,6 +7014,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="J6" r:id="rId1" location="" tooltip="" display="bill.com"/>
+    <hyperlink ref="J26" r:id="rId2" location="" tooltip="" display="bill.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
@@ -6902,37 +7047,37 @@
         <v>65</v>
       </c>
       <c r="B1" t="s" s="39">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="C1" t="s" s="39">
         <v>55</v>
       </c>
       <c r="D1" t="s" s="39">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="E1" t="s" s="39">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="F1" t="s" s="39">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="G1" t="s" s="39">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="H1" t="s" s="39">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="I1" t="s" s="39">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="J1" t="s" s="39">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="K1" t="s" s="39">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="L1" t="s" s="39">
-        <v>364</v>
+        <v>376</v>
       </c>
       <c r="M1" t="s" s="39">
         <v>66</v>
@@ -6940,89 +7085,89 @@
     </row>
     <row r="2" ht="90" customHeight="1">
       <c r="A2" t="s" s="40">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B2" t="s" s="31">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C2" t="s" s="40">
         <v>67</v>
       </c>
       <c r="D2" t="s" s="40">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="E2" t="s" s="31">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="F2" t="s" s="31">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="G2" t="s" s="31">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="H2" s="55">
         <v>5</v>
       </c>
       <c r="I2" t="s" s="40">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="J2" t="s" s="40">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="K2" t="s" s="40">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="L2" t="s" s="40">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="M2" t="s" s="40">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1">
       <c r="A3" t="s" s="40">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="B3" t="s" s="31">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="C3" t="s" s="40">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="D3" t="s" s="40">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="E3" t="s" s="31">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="F3" t="s" s="31">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="G3" t="s" s="31">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="H3" s="55">
         <v>4</v>
       </c>
       <c r="I3" t="s" s="40">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="J3" t="s" s="40">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="K3" t="s" s="40">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="L3" t="s" s="40">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="M3" t="s" s="40">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" ht="12.7" customHeight="1">
       <c r="A4" t="s" s="56">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="B4" s="57"/>
       <c r="C4" s="57"/>
@@ -7189,7 +7334,7 @@
     <row r="2" ht="27.75" customHeight="1">
       <c r="A2" s="7"/>
       <c r="B2" t="s" s="9">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="C2" s="21"/>
       <c r="D2" s="21"/>
@@ -7201,7 +7346,7 @@
     <row r="3" ht="13.55" customHeight="1">
       <c r="A3" s="7"/>
       <c r="B3" t="s" s="10">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="C3" s="60"/>
       <c r="D3" s="60"/>
@@ -7223,7 +7368,7 @@
     <row r="5" ht="17.55" customHeight="1">
       <c r="A5" s="7"/>
       <c r="B5" t="s" s="61">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="C5" s="62"/>
       <c r="D5" s="62"/>
@@ -7241,19 +7386,19 @@
         <v>55</v>
       </c>
       <c r="D6" t="s" s="39">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="E6" t="s" s="39">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="F6" t="s" s="39">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="G6" t="s" s="39">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="H6" t="s" s="39">
-        <v>392</v>
+        <v>404</v>
       </c>
     </row>
     <row r="7" ht="25.5" customHeight="1">
@@ -7266,31 +7411,31 @@
       </c>
       <c r="D7" s="65" cm="1">
         <f t="array" ref="D7">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"GV",'CSF Scoring'!G1:G107),"")</f>
-        <v>1.78947368421053</v>
+        <v>1.54838709677419</v>
       </c>
       <c r="E7" s="65" cm="1">
         <f t="array" ref="E7">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"GV",'CSF Scoring'!H1:H107),"")</f>
-        <v>2.94736842105263</v>
+        <v>2.96774193548387</v>
       </c>
       <c r="F7" s="65" cm="1">
         <f t="array" ref="F7">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"GV",'CSF Scoring'!I1:I107),"")</f>
-        <v>1.15789473684211</v>
+        <v>1.41935483870968</v>
       </c>
       <c r="G7" s="66" cm="1">
         <f t="array" ref="G7">_xlfn.COUNTIFS('CSF Scoring'!B1:B107,"GV",'CSF Scoring'!G1:G107,"&gt;0")/COUNTIF('CSF Scoring'!B1:B107,"GV")</f>
-        <v>0.612903225806452</v>
+        <v>1</v>
       </c>
       <c r="H7" t="s" s="67">
-        <v>393</v>
+        <v>405</v>
       </c>
     </row>
     <row r="8" ht="25.5" customHeight="1">
       <c r="A8" s="14"/>
       <c r="B8" t="s" s="68">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C8" t="s" s="17">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D8" t="str" s="44" cm="1">
         <f t="array" ref="D8">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"ID",'CSF Scoring'!G1:G107),"")</f>
@@ -7306,16 +7451,16 @@
         <v>0</v>
       </c>
       <c r="H8" t="s" s="67">
-        <v>394</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" ht="25.5" customHeight="1">
       <c r="A9" s="14"/>
       <c r="B9" t="s" s="69">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C9" t="s" s="17">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="D9" t="str" s="44" cm="1">
         <f t="array" ref="D9">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"PR",'CSF Scoring'!G1:G107),"")</f>
@@ -7331,16 +7476,16 @@
         <v>0</v>
       </c>
       <c r="H9" t="s" s="67">
-        <v>395</v>
+        <v>407</v>
       </c>
     </row>
     <row r="10" ht="25.5" customHeight="1">
       <c r="A10" s="14"/>
       <c r="B10" t="s" s="70">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C10" t="s" s="17">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="D10" t="str" s="44" cm="1">
         <f t="array" ref="D10">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"DE",'CSF Scoring'!G1:G107),"")</f>
@@ -7356,16 +7501,16 @@
         <v>0</v>
       </c>
       <c r="H10" t="s" s="67">
-        <v>396</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" ht="25.5" customHeight="1">
       <c r="A11" s="14"/>
       <c r="B11" t="s" s="71">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C11" t="s" s="17">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="D11" t="str" s="44" cm="1">
         <f t="array" ref="D11">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"RS",'CSF Scoring'!G1:G107),"")</f>
@@ -7381,16 +7526,16 @@
         <v>0</v>
       </c>
       <c r="H11" t="s" s="67">
-        <v>397</v>
+        <v>409</v>
       </c>
     </row>
     <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="14"/>
       <c r="B12" t="s" s="72">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C12" t="s" s="73">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="D12" t="str" s="74" cm="1">
         <f t="array" ref="D12">_xlfn.IFERROR(_xlfn.AVERAGEIF('CSF Scoring'!B1:B107,"RC",'CSF Scoring'!G1:G107),"")</f>
@@ -7406,35 +7551,35 @@
         <v>0</v>
       </c>
       <c r="H12" t="s" s="76">
-        <v>398</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="63"/>
       <c r="B13" t="s" s="77">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="C13" t="s" s="78">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="D13" s="79" cm="1">
         <f t="array" ref="D13">_xlfn.IFERROR(AVERAGE('CSF Scoring'!G2:G107),"")</f>
-        <v>1.78947368421053</v>
+        <v>1.54838709677419</v>
       </c>
       <c r="E13" s="79" cm="1">
         <f t="array" ref="E13">_xlfn.IFERROR(AVERAGE('CSF Scoring'!H2:H107),"")</f>
-        <v>2.94736842105263</v>
+        <v>2.96774193548387</v>
       </c>
       <c r="F13" s="79" cm="1">
         <f t="array" ref="F13">_xlfn.IFERROR(AVERAGE('CSF Scoring'!I2:I107),"")</f>
-        <v>1.15789473684211</v>
+        <v>1.41935483870968</v>
       </c>
       <c r="G13" s="80" cm="1">
         <f t="array" ref="G13">COUNTIF('CSF Scoring'!G2:G107,"&gt;0")/106</f>
-        <v>0.179245283018868</v>
+        <v>0.292452830188679</v>
       </c>
       <c r="H13" t="s" s="78">
-        <v>401</v>
+        <v>413</v>
       </c>
     </row>
     <row r="14" ht="13.55" customHeight="1">
@@ -7450,7 +7595,7 @@
     <row r="15" ht="17.55" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" t="s" s="61">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="C15" s="62"/>
       <c r="D15" s="62"/>
@@ -7462,16 +7607,16 @@
     <row r="16" ht="21.75" customHeight="1">
       <c r="A16" s="63"/>
       <c r="B16" t="s" s="39">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="C16" t="s" s="39">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="D16" t="s" s="39">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="E16" t="s" s="39">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="F16" s="82"/>
       <c r="G16" s="7"/>
@@ -7483,7 +7628,7 @@
         <v>0</v>
       </c>
       <c r="C17" t="s" s="84">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="D17" s="85" cm="1">
         <f t="array" ref="D17">COUNTIF('CSF Scoring'!I2:I107,0)</f>
@@ -7491,7 +7636,7 @@
       </c>
       <c r="E17" s="86" cm="1">
         <f t="array" ref="E17">_xlfn.IFERROR(D17/COUNT('CSF Scoring'!I2:I107),"")</f>
-        <v>0.105263157894737</v>
+        <v>0.0645161290322581</v>
       </c>
       <c r="F17" s="87"/>
       <c r="G17" s="7"/>
@@ -7503,15 +7648,15 @@
         <v>1</v>
       </c>
       <c r="C18" t="s" s="89">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D18" s="55" cm="1">
         <f t="array" ref="D18">COUNTIF('CSF Scoring'!I2:I107,1)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E18" s="90" cm="1">
         <f t="array" ref="E18">_xlfn.IFERROR(D18/COUNT('CSF Scoring'!I2:I107),"")</f>
-        <v>0.631578947368421</v>
+        <v>0.451612903225806</v>
       </c>
       <c r="F18" s="87"/>
       <c r="G18" s="7"/>
@@ -7523,15 +7668,15 @@
         <v>2</v>
       </c>
       <c r="C19" t="s" s="92">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="D19" s="93" cm="1">
         <f t="array" ref="D19">COUNTIF('CSF Scoring'!I2:I107,2)</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E19" s="94" cm="1">
         <f t="array" ref="E19">_xlfn.IFERROR(D19/COUNT('CSF Scoring'!I2:I107),"")</f>
-        <v>0.263157894736842</v>
+        <v>0.483870967741935</v>
       </c>
       <c r="F19" s="87"/>
       <c r="G19" s="7"/>
@@ -7543,7 +7688,7 @@
         <v>3</v>
       </c>
       <c r="C20" t="s" s="96">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="D20" s="97" cm="1">
         <f t="array" ref="D20">COUNTIF('CSF Scoring'!I2:I107,3)</f>
@@ -7570,7 +7715,7 @@
     <row r="22" ht="17.55" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" t="s" s="61">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="C22" s="62"/>
       <c r="D22" s="62"/>
@@ -7588,10 +7733,10 @@
         <v>32</v>
       </c>
       <c r="D23" t="s" s="39">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="E23" t="s" s="39">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="F23" s="82"/>
       <c r="G23" s="7"/>
@@ -7607,11 +7752,11 @@
       </c>
       <c r="D24" s="97" cm="1">
         <f t="array" ref="D24">COUNTIF('CSF Scoring'!G2:G107,1)</f>
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E24" s="98" cm="1">
         <f t="array" ref="E24">_xlfn.IFERROR(D24/COUNT('CSF Scoring'!G2:G107),"")</f>
-        <v>0.315789473684211</v>
+        <v>0.5161290322580649</v>
       </c>
       <c r="F24" s="87"/>
       <c r="G24" s="7"/>
@@ -7627,11 +7772,11 @@
       </c>
       <c r="D25" s="93" cm="1">
         <f t="array" ref="D25">COUNTIF('CSF Scoring'!G2:G107,2)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E25" s="94" cm="1">
         <f t="array" ref="E25">_xlfn.IFERROR(D25/COUNT('CSF Scoring'!G2:G107),"")</f>
-        <v>0.578947368421053</v>
+        <v>0.419354838709677</v>
       </c>
       <c r="F25" s="87"/>
       <c r="G25" s="7"/>
@@ -7651,7 +7796,7 @@
       </c>
       <c r="E26" s="90" cm="1">
         <f t="array" ref="E26">_xlfn.IFERROR(D26/COUNT('CSF Scoring'!G2:G107),"")</f>
-        <v>0.105263157894737</v>
+        <v>0.0645161290322581</v>
       </c>
       <c r="F26" s="87"/>
       <c r="G26" s="7"/>

</xml_diff>